<commit_message>
docs: clarify workflow positioning and samples
</commit_message>
<xml_diff>
--- a/site/examples/sample-raw.xlsx
+++ b/site/examples/sample-raw.xlsx
@@ -11,27 +11,27 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
-  <si>
-    <t>Customer</t>
-  </si>
-  <si>
-    <t>Amount</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
+  <si>
+    <t>Account</t>
   </si>
   <si>
     <t>Region</t>
   </si>
   <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Acme Co</t>
+    <t>Renewal</t>
+  </si>
+  <si>
+    <t>Owner</t>
+  </si>
+  <si>
+    <t>Acme Logistics</t>
   </si>
   <si>
     <t>Seoul</t>
   </si>
   <si>
-    <t>VIP</t>
+    <t>Mina</t>
   </si>
   <si>
     <t>Beta Works</t>
@@ -40,7 +40,7 @@
     <t>Busan</t>
   </si>
   <si>
-    <t>Standard</t>
+    <t>Joon</t>
   </si>
   <si>
     <t>Core Labs</t>
@@ -49,10 +49,22 @@
     <t>Daejeon</t>
   </si>
   <si>
-    <t>Delta Mart</t>
+    <t>Hana</t>
+  </si>
+  <si>
+    <t>Delta Retail</t>
   </si>
   <si>
     <t>Incheon</t>
+  </si>
+  <si>
+    <t>Sol</t>
+  </si>
+  <si>
+    <t>Evergreen Foods</t>
+  </si>
+  <si>
+    <t>Gwangju</t>
   </si>
 </sst>
 </file>
@@ -85,7 +97,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -93,19 +105,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF185C37"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -445,26 +463,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="14" style="1" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -472,11 +489,11 @@
       <c r="A2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="1">
-        <v>1200</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B2" t="s">
         <v>5</v>
+      </c>
+      <c r="C2" s="2">
+        <v>18400</v>
       </c>
       <c r="D2" t="s">
         <v>6</v>
@@ -486,11 +503,11 @@
       <c r="A3" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="1">
-        <v>350</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="B3" t="s">
         <v>8</v>
+      </c>
+      <c r="C3" s="2">
+        <v>7200</v>
       </c>
       <c r="D3" t="s">
         <v>9</v>
@@ -500,27 +517,41 @@
       <c r="A4" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="1">
-        <v>820</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="B4" t="s">
         <v>11</v>
       </c>
+      <c r="C4" s="2">
+        <v>12600</v>
+      </c>
       <c r="D4" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="1">
-        <v>1560</v>
-      </c>
-      <c r="C5" t="s">
         <v>13</v>
       </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="2">
+        <v>9800</v>
+      </c>
       <c r="D5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="2">
+        <v>21300</v>
+      </c>
+      <c r="D6" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>